<commit_message>
Converting clean.xlsx to csv, adding first steps to Quarto
</commit_message>
<xml_diff>
--- a/data/processed/clean.xlsx
+++ b/data/processed/clean.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Startklar\Desktop\UrbanFledgling\data\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44672023-1F19-4F8C-A148-76452EB7C04C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19049B79-7474-486A-A905-E57389FEB9FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3C6DA8FA-A6A7-461C-899B-42C5129D3C48}"/>
+    <workbookView xWindow="9564" yWindow="612" windowWidth="13476" windowHeight="10980" activeTab="1" xr2:uid="{3C6DA8FA-A6A7-461C-899B-42C5129D3C48}"/>
   </bookViews>
   <sheets>
     <sheet name="UrbanFledglings" sheetId="1" r:id="rId1"/>
+    <sheet name="Code Book" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
   <si>
     <t>15 - 17</t>
   </si>
@@ -41,6 +42,39 @@
   </si>
   <si>
     <t>environmental_noise_dB</t>
+  </si>
+  <si>
+    <t>variable</t>
+  </si>
+  <si>
+    <t>Definition</t>
+  </si>
+  <si>
+    <t>possible values</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>num</t>
+  </si>
+  <si>
+    <t>chr</t>
+  </si>
+  <si>
+    <t>English</t>
+  </si>
+  <si>
+    <t>Number of urband fledglings found in a nest.</t>
+  </si>
+  <si>
+    <t>Insect abundance in the nest in g/m^2</t>
+  </si>
+  <si>
+    <t>Environmental noise near the nest measured in dB</t>
+  </si>
+  <si>
+    <t>Additional comments about the data</t>
   </si>
 </sst>
 </file>
@@ -589,10 +623,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1384,4 +1414,89 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{501FDC9F-802A-486E-AFAF-C14B27B350E8}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="23.33203125" customWidth="1"/>
+    <col min="2" max="2" width="38.88671875" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>